<commit_message>
feat: implement ₹120 Cr purse limit enforcement in auction panels and sync results
</commit_message>
<xml_diff>
--- a/auction_results.xlsx
+++ b/auction_results.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,35 +415,21 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Rohit Sharma</v>
+        <v>Suryakumar Yadav</v>
       </c>
       <c r="B2" t="str">
         <v>MI</v>
       </c>
       <c r="C2" t="str">
-        <v>₹600,00,000</v>
+        <v>₹1400,00,000</v>
       </c>
       <c r="D2">
         <v>10</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Mohammed Shami</v>
-      </c>
-      <c r="B3" t="str">
-        <v>KKR</v>
-      </c>
-      <c r="C3" t="str">
-        <v>₹700,00,000</v>
-      </c>
-      <c r="D3">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: expand mock stats for more players
</commit_message>
<xml_diff>
--- a/auction_results.xlsx
+++ b/auction_results.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,21 +415,49 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Suryakumar Yadav</v>
+        <v>Rohit Sharma</v>
       </c>
       <c r="B2" t="str">
+        <v>CSK</v>
+      </c>
+      <c r="C2" t="str">
+        <v>₹250,00,000</v>
+      </c>
+      <c r="D2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Hardik Pandya</v>
+      </c>
+      <c r="B3" t="str">
         <v>MI</v>
       </c>
-      <c r="C2" t="str">
-        <v>₹1400,00,000</v>
-      </c>
-      <c r="D2">
+      <c r="C3" t="str">
+        <v>₹1500,00,000</v>
+      </c>
+      <c r="D3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Virat Kohli</v>
+      </c>
+      <c r="B4" t="str">
+        <v>MI</v>
+      </c>
+      <c r="C4" t="str">
+        <v>₹1500,00,000</v>
+      </c>
+      <c r="D4">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add player search functionality to catalog
</commit_message>
<xml_diff>
--- a/auction_results.xlsx
+++ b/auction_results.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,49 +415,21 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Rohit Sharma</v>
+        <v>Suryakumar Yadav</v>
       </c>
       <c r="B2" t="str">
         <v>CSK</v>
       </c>
       <c r="C2" t="str">
-        <v>₹250,00,000</v>
+        <v>₹700,00,000</v>
       </c>
       <c r="D2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Hardik Pandya</v>
-      </c>
-      <c r="B3" t="str">
-        <v>MI</v>
-      </c>
-      <c r="C3" t="str">
-        <v>₹1500,00,000</v>
-      </c>
-      <c r="D3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Virat Kohli</v>
-      </c>
-      <c r="B4" t="str">
-        <v>MI</v>
-      </c>
-      <c r="C4" t="str">
-        <v>₹1500,00,000</v>
-      </c>
-      <c r="D4">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: update auction results
</commit_message>
<xml_diff>
--- a/auction_results.xlsx
+++ b/auction_results.xlsx
@@ -415,13 +415,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Suryakumar Yadav</v>
+        <v>Hardik Pandya</v>
       </c>
       <c r="B2" t="str">
         <v>CSK</v>
       </c>
       <c r="C2" t="str">
-        <v>₹700,00,000</v>
+        <v>₹2,00,000</v>
       </c>
       <c r="D2">
         <v>10</v>

</xml_diff>

<commit_message>
feat: lock anonymous bids and display timestamp
</commit_message>
<xml_diff>
--- a/auction_results.xlsx
+++ b/auction_results.xlsx
@@ -418,10 +418,10 @@
         <v>Hardik Pandya</v>
       </c>
       <c r="B2" t="str">
-        <v>CSK</v>
+        <v>MI</v>
       </c>
       <c r="C2" t="str">
-        <v>₹2,00,000</v>
+        <v>₹10,80,00,000</v>
       </c>
       <c r="D2">
         <v>10</v>

</xml_diff>